<commit_message>
Add BANREP inflation and Brent pipelines
Introduce BANREP (SUAMECA) inflation and FRED/EIA Brent pipelines: add orchestration scripts (run_banrep_inflation.py, run_brent.py), new source/raw fixtures (banrep JSON, fred CSV) and processed outputs (inflation_banrep_colombia.csv, brent_colombia.csv). Update orchestration (run_all.py, src/main.py) and quality checks to handle new series, add tests for BANREP and Brent, and adjust existing GEIH/IPC files and tests. Refresh README to document new data sources, outputs, test counts and usage. This integrates inflation and oil-price series into the reproducible NAIRU pipeline and adds offline fixtures for CI.
</commit_message>
<xml_diff>
--- a/data/raw/dane/ipc_indices_raw.xlsx
+++ b/data/raw/dane/ipc_indices_raw.xlsx
@@ -72,7 +72,7 @@
       <rPr>
         <b/>
         <sz val="8"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Segoe UI"/>
         <family val="2"/>
       </rPr>
@@ -81,7 +81,7 @@
     <r>
       <rPr>
         <sz val="8"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Segoe UI"/>
         <family val="2"/>
       </rPr>
@@ -96,7 +96,7 @@
       <rPr>
         <b/>
         <sz val="8"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Segoe UI"/>
         <family val="2"/>
       </rPr>
@@ -105,7 +105,7 @@
     <r>
       <rPr>
         <sz val="8"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Segoe UI"/>
         <family val="2"/>
       </rPr>
@@ -121,7 +121,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -131,8 +131,14 @@
     </font>
     <font>
       <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
@@ -145,27 +151,27 @@
     <font>
       <b/>
       <sz val="12"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="8"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
@@ -516,7 +522,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="60">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -525,163 +531,175 @@
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="5" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="5" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="5" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="6" applyBorder="1" fontId="5" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="6" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="7" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="8" applyBorder="1" fontId="5" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="9" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="9" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="11" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="12" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="13" applyBorder="1" fontId="5" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="14" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="15" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="12" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="16" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="17" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="18" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="19" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="20" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="21" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="22" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="23" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="24" applyBorder="1" fontId="6" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="7" applyBorder="1" fontId="6" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="8" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="6" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="18" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="22" applyBorder="1" fontId="7" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="7" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="7" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="23" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="4" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="4" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="6" applyBorder="1" fontId="4" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="6" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="7" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="8" applyBorder="1" fontId="4" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="9" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="9" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="11" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="12" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="13" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="14" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="15" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="12" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="16" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="17" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="18" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="19" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="20" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="21" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="22" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="23" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="24" applyBorder="1" fontId="5" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="7" applyBorder="1" fontId="5" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="8" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="5" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="18" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="22" applyBorder="1" fontId="6" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="6" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="6" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="23" applyBorder="1" fontId="1" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -988,33 +1006,33 @@
   <dimension ref="A1:AA26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="53" width="23.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="54" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="54" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="54" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="54" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="54" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="54" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="55" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="54" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="54" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="54" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="54" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="54" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="54" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="54" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="54" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="54" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="54" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="54" width="8.005" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="54" width="8.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="54" width="8.005" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="54" width="8.005" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="54" width="8.005" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="54" width="8.005" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="54" width="8.005" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="53" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="27" max="27" style="53" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="55" width="23.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="56" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="56" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="56" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="56" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="56" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="56" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="57" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="56" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="56" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="56" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="56" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="56" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="56" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="56" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="56" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="56" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="56" width="7.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="56" width="8.005" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="57" width="8.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="57" width="8.005" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="57" width="8.005" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="57" width="8.005" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="57" width="8.005" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="57" width="8.005" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="58" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="59" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25">
@@ -1044,459 +1062,459 @@
       <c r="X1" s="2"/>
       <c r="Y1" s="2"/>
       <c r="Z1" s="3"/>
-      <c r="AA1" s="3"/>
+      <c r="AA1" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
-      <c r="A2" s="3"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="4"/>
-      <c r="Q2" s="4"/>
-      <c r="R2" s="4"/>
-      <c r="S2" s="4"/>
-      <c r="T2" s="4"/>
-      <c r="U2" s="4"/>
-      <c r="V2" s="4"/>
-      <c r="W2" s="4"/>
-      <c r="X2" s="4"/>
-      <c r="Y2" s="4"/>
+      <c r="A2" s="5"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6"/>
+      <c r="S2" s="6"/>
+      <c r="T2" s="6"/>
+      <c r="U2" s="6"/>
+      <c r="V2" s="6"/>
+      <c r="W2" s="6"/>
+      <c r="X2" s="6"/>
+      <c r="Y2" s="6"/>
       <c r="Z2" s="3"/>
-      <c r="AA2" s="3"/>
+      <c r="AA2" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
-      <c r="L3" s="7"/>
-      <c r="M3" s="7"/>
-      <c r="N3" s="7"/>
-      <c r="O3" s="7"/>
-      <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
-      <c r="R3" s="7"/>
-      <c r="S3" s="7"/>
-      <c r="T3" s="7"/>
-      <c r="U3" s="7"/>
-      <c r="V3" s="7"/>
-      <c r="W3" s="7"/>
-      <c r="X3" s="7"/>
-      <c r="Y3" s="7"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9"/>
+      <c r="S3" s="9"/>
+      <c r="T3" s="9"/>
+      <c r="U3" s="9"/>
+      <c r="V3" s="9"/>
+      <c r="W3" s="9"/>
+      <c r="X3" s="9"/>
+      <c r="Y3" s="9"/>
       <c r="Z3" s="3"/>
-      <c r="AA3" s="3"/>
+      <c r="AA3" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
-      <c r="A4" s="8"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="7"/>
-      <c r="M4" s="7"/>
-      <c r="N4" s="7"/>
-      <c r="O4" s="7"/>
-      <c r="P4" s="7"/>
-      <c r="Q4" s="7"/>
-      <c r="R4" s="7"/>
-      <c r="S4" s="7"/>
-      <c r="T4" s="7"/>
-      <c r="U4" s="7"/>
-      <c r="V4" s="7"/>
-      <c r="W4" s="7"/>
-      <c r="X4" s="7"/>
-      <c r="Y4" s="7"/>
+      <c r="A4" s="10"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="9"/>
+      <c r="P4" s="9"/>
+      <c r="Q4" s="9"/>
+      <c r="R4" s="9"/>
+      <c r="S4" s="9"/>
+      <c r="T4" s="9"/>
+      <c r="U4" s="9"/>
+      <c r="V4" s="9"/>
+      <c r="W4" s="9"/>
+      <c r="X4" s="9"/>
+      <c r="Y4" s="9"/>
       <c r="Z4" s="3"/>
-      <c r="AA4" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="33.75" customFormat="1" s="9">
-      <c r="A5" s="10" t="s">
+      <c r="AA4" s="4"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="33.75" customFormat="1" s="11">
+      <c r="A5" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11"/>
-      <c r="O5" s="11"/>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="11"/>
-      <c r="R5" s="11"/>
-      <c r="S5" s="11"/>
-      <c r="T5" s="11"/>
-      <c r="U5" s="11"/>
-      <c r="V5" s="11"/>
-      <c r="W5" s="11"/>
-      <c r="X5" s="11"/>
-      <c r="Y5" s="11"/>
-      <c r="Z5" s="12"/>
-      <c r="AA5" s="12"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+      <c r="I5" s="13"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="13"/>
+      <c r="L5" s="13"/>
+      <c r="M5" s="13"/>
+      <c r="N5" s="13"/>
+      <c r="O5" s="13"/>
+      <c r="P5" s="13"/>
+      <c r="Q5" s="13"/>
+      <c r="R5" s="13"/>
+      <c r="S5" s="13"/>
+      <c r="T5" s="13"/>
+      <c r="U5" s="13"/>
+      <c r="V5" s="13"/>
+      <c r="W5" s="13"/>
+      <c r="X5" s="13"/>
+      <c r="Y5" s="13"/>
+      <c r="Z5" s="14"/>
+      <c r="AA5" s="14"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
-      <c r="A6" s="3"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
-      <c r="M6" s="4"/>
-      <c r="N6" s="4"/>
-      <c r="O6" s="4"/>
-      <c r="P6" s="4"/>
-      <c r="Q6" s="4"/>
-      <c r="R6" s="4"/>
-      <c r="S6" s="4"/>
-      <c r="T6" s="4"/>
-      <c r="U6" s="4"/>
-      <c r="V6" s="4"/>
-      <c r="W6" s="4"/>
-      <c r="X6" s="4"/>
-      <c r="Y6" s="4"/>
+      <c r="A6" s="5"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="6"/>
+      <c r="T6" s="6"/>
+      <c r="U6" s="6"/>
+      <c r="V6" s="6"/>
+      <c r="W6" s="6"/>
+      <c r="X6" s="6"/>
+      <c r="Y6" s="6"/>
       <c r="Z6" s="3"/>
-      <c r="AA6" s="3"/>
+      <c r="AA6" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
-      <c r="A7" s="13"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="14"/>
-      <c r="J7" s="14"/>
-      <c r="K7" s="14"/>
-      <c r="L7" s="14"/>
-      <c r="M7" s="14"/>
-      <c r="N7" s="14"/>
-      <c r="O7" s="14"/>
-      <c r="P7" s="14"/>
-      <c r="Q7" s="14"/>
-      <c r="R7" s="14"/>
-      <c r="S7" s="15"/>
-      <c r="T7" s="14"/>
-      <c r="U7" s="14"/>
-      <c r="V7" s="14"/>
-      <c r="W7" s="14"/>
-      <c r="X7" s="14"/>
-      <c r="Y7" s="14"/>
+      <c r="A7" s="15"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="16"/>
+      <c r="P7" s="16"/>
+      <c r="Q7" s="16"/>
+      <c r="R7" s="16"/>
+      <c r="S7" s="17"/>
+      <c r="T7" s="16"/>
+      <c r="U7" s="16"/>
+      <c r="V7" s="16"/>
+      <c r="W7" s="16"/>
+      <c r="X7" s="16"/>
+      <c r="Y7" s="16"/>
       <c r="Z7" s="3"/>
-      <c r="AA7" s="3"/>
+      <c r="AA7" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
-      <c r="A8" s="16"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="17"/>
-      <c r="M8" s="17"/>
-      <c r="N8" s="17"/>
-      <c r="O8" s="17"/>
-      <c r="P8" s="17"/>
-      <c r="Q8" s="17"/>
-      <c r="R8" s="17"/>
-      <c r="S8" s="17"/>
-      <c r="T8" s="18"/>
-      <c r="U8" s="19"/>
-      <c r="V8" s="18"/>
-      <c r="W8" s="19"/>
-      <c r="X8" s="19"/>
-      <c r="Y8" s="20" t="s">
+      <c r="A8" s="18"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="19"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="19"/>
+      <c r="N8" s="19"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="19"/>
+      <c r="Q8" s="19"/>
+      <c r="R8" s="19"/>
+      <c r="S8" s="19"/>
+      <c r="T8" s="20"/>
+      <c r="U8" s="21"/>
+      <c r="V8" s="20"/>
+      <c r="W8" s="21"/>
+      <c r="X8" s="21"/>
+      <c r="Y8" s="22" t="s">
         <v>2</v>
       </c>
       <c r="Z8" s="3"/>
-      <c r="AA8" s="3"/>
+      <c r="AA8" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="17.25">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="22">
+      <c r="B9" s="24">
         <v>2003</v>
       </c>
-      <c r="C9" s="23">
+      <c r="C9" s="25">
         <v>2004</v>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="25">
         <v>2005</v>
       </c>
-      <c r="E9" s="23">
+      <c r="E9" s="25">
         <v>2006</v>
       </c>
-      <c r="F9" s="23">
+      <c r="F9" s="25">
         <v>2007</v>
       </c>
-      <c r="G9" s="23">
+      <c r="G9" s="25">
         <v>2008</v>
       </c>
-      <c r="H9" s="23">
+      <c r="H9" s="25">
         <v>2009</v>
       </c>
-      <c r="I9" s="23">
+      <c r="I9" s="25">
         <v>2010</v>
       </c>
-      <c r="J9" s="23">
+      <c r="J9" s="25">
         <v>2011</v>
       </c>
-      <c r="K9" s="23">
+      <c r="K9" s="25">
         <v>2012</v>
       </c>
-      <c r="L9" s="23">
+      <c r="L9" s="25">
         <v>2013</v>
       </c>
-      <c r="M9" s="23">
+      <c r="M9" s="25">
         <v>2014</v>
       </c>
-      <c r="N9" s="23">
+      <c r="N9" s="25">
         <v>2015</v>
       </c>
-      <c r="O9" s="23">
+      <c r="O9" s="25">
         <v>2016</v>
       </c>
-      <c r="P9" s="23">
+      <c r="P9" s="25">
         <v>2017</v>
       </c>
-      <c r="Q9" s="23">
+      <c r="Q9" s="25">
         <v>2018</v>
       </c>
-      <c r="R9" s="23">
+      <c r="R9" s="25">
         <v>2019</v>
       </c>
-      <c r="S9" s="24">
+      <c r="S9" s="26">
         <v>2020</v>
       </c>
-      <c r="T9" s="24">
+      <c r="T9" s="26">
         <v>2021</v>
       </c>
-      <c r="U9" s="24">
+      <c r="U9" s="26">
         <v>2022</v>
       </c>
-      <c r="V9" s="25">
+      <c r="V9" s="27">
         <v>2023</v>
       </c>
-      <c r="W9" s="25">
+      <c r="W9" s="27">
         <v>2024</v>
       </c>
-      <c r="X9" s="25">
+      <c r="X9" s="27">
         <v>2025</v>
       </c>
-      <c r="Y9" s="26">
+      <c r="Y9" s="28">
         <v>2026</v>
       </c>
       <c r="Z9" s="3"/>
-      <c r="AA9" s="3"/>
+      <c r="AA9" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="17.25">
-      <c r="A10" s="27" t="s">
+      <c r="A10" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="28">
+      <c r="B10" s="30">
         <v>50.42</v>
       </c>
-      <c r="C10" s="29">
+      <c r="C10" s="31">
         <v>53.54</v>
       </c>
-      <c r="D10" s="29">
+      <c r="D10" s="31">
         <v>56.45</v>
       </c>
-      <c r="E10" s="29">
+      <c r="E10" s="31">
         <v>59.02</v>
       </c>
-      <c r="F10" s="29">
+      <c r="F10" s="31">
         <v>61.8</v>
       </c>
-      <c r="G10" s="29">
+      <c r="G10" s="31">
         <v>65.51</v>
       </c>
-      <c r="H10" s="29">
+      <c r="H10" s="31">
         <v>70.21</v>
       </c>
-      <c r="I10" s="29">
+      <c r="I10" s="31">
         <v>71.69</v>
       </c>
-      <c r="J10" s="29">
+      <c r="J10" s="31">
         <v>74.12</v>
       </c>
-      <c r="K10" s="29">
+      <c r="K10" s="31">
         <v>76.75</v>
       </c>
-      <c r="L10" s="29">
+      <c r="L10" s="31">
         <v>78.28</v>
       </c>
-      <c r="M10" s="29">
+      <c r="M10" s="31">
         <v>79.95</v>
       </c>
-      <c r="N10" s="29">
+      <c r="N10" s="31">
         <v>83</v>
       </c>
-      <c r="O10" s="29">
+      <c r="O10" s="31">
         <v>89.19</v>
       </c>
-      <c r="P10" s="29">
+      <c r="P10" s="31">
         <v>94.07</v>
       </c>
-      <c r="Q10" s="29">
+      <c r="Q10" s="31">
         <v>97.53</v>
       </c>
-      <c r="R10" s="29">
+      <c r="R10" s="31">
         <v>100.6</v>
       </c>
-      <c r="S10" s="29">
+      <c r="S10" s="31">
         <v>104.24</v>
       </c>
-      <c r="T10" s="29">
+      <c r="T10" s="31">
         <v>105.91</v>
       </c>
-      <c r="U10" s="29">
+      <c r="U10" s="31">
         <v>113.26</v>
       </c>
-      <c r="V10" s="29">
+      <c r="V10" s="31">
         <v>128.27</v>
       </c>
-      <c r="W10" s="29">
+      <c r="W10" s="31">
         <v>138.98</v>
       </c>
-      <c r="X10" s="29">
+      <c r="X10" s="31">
         <v>146.24</v>
       </c>
-      <c r="Y10" s="30">
+      <c r="Y10" s="32">
         <v>154.07</v>
       </c>
       <c r="Z10" s="3"/>
-      <c r="AA10" s="3"/>
+      <c r="AA10" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="17.25">
-      <c r="A11" s="31" t="s">
+      <c r="A11" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="32">
+      <c r="B11" s="34">
         <v>50.98</v>
       </c>
-      <c r="C11" s="33">
+      <c r="C11" s="35">
         <v>54.18</v>
       </c>
-      <c r="D11" s="33">
+      <c r="D11" s="35">
         <v>57.02</v>
       </c>
-      <c r="E11" s="33">
+      <c r="E11" s="35">
         <v>59.41</v>
       </c>
-      <c r="F11" s="33">
+      <c r="F11" s="35">
         <v>62.53</v>
       </c>
-      <c r="G11" s="33">
+      <c r="G11" s="35">
         <v>66.5</v>
       </c>
-      <c r="H11" s="33">
+      <c r="H11" s="35">
         <v>70.8</v>
       </c>
-      <c r="I11" s="33">
+      <c r="I11" s="35">
         <v>72.28</v>
       </c>
-      <c r="J11" s="33">
+      <c r="J11" s="35">
         <v>74.57</v>
       </c>
-      <c r="K11" s="33">
+      <c r="K11" s="35">
         <v>77.22</v>
       </c>
-      <c r="L11" s="33">
+      <c r="L11" s="35">
         <v>78.63</v>
       </c>
-      <c r="M11" s="33">
+      <c r="M11" s="35">
         <v>80.45</v>
       </c>
-      <c r="N11" s="33">
+      <c r="N11" s="35">
         <v>83.96</v>
       </c>
-      <c r="O11" s="33">
+      <c r="O11" s="35">
         <v>90.33</v>
       </c>
-      <c r="P11" s="33">
+      <c r="P11" s="35">
         <v>95.01</v>
       </c>
-      <c r="Q11" s="33">
+      <c r="Q11" s="35">
         <v>98.22</v>
       </c>
-      <c r="R11" s="33">
+      <c r="R11" s="35">
         <v>101.18</v>
       </c>
-      <c r="S11" s="33">
+      <c r="S11" s="35">
         <v>104.94</v>
       </c>
-      <c r="T11" s="33">
+      <c r="T11" s="35">
         <v>106.58</v>
       </c>
-      <c r="U11" s="33">
+      <c r="U11" s="35">
         <v>115.11</v>
       </c>
-      <c r="V11" s="33">
+      <c r="V11" s="35">
         <v>130.4</v>
       </c>
-      <c r="W11" s="33">
+      <c r="W11" s="35">
         <v>140.49</v>
       </c>
-      <c r="X11" s="33">
+      <c r="X11" s="35">
         <v>147.9</v>
       </c>
-      <c r="Y11" s="34">
+      <c r="Y11" s="36">
         <v>155.73</v>
       </c>
       <c r="Z11" s="3"/>
-      <c r="AA11" s="3"/>
+      <c r="AA11" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="17.25">
-      <c r="A12" s="27" t="s">
+      <c r="A12" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="35">
+      <c r="B12" s="37">
         <v>51.51</v>
       </c>
       <c r="C12" s="2">
@@ -1565,92 +1583,92 @@
       <c r="X12" s="2">
         <v>148.68</v>
       </c>
-      <c r="Y12" s="36"/>
+      <c r="Y12" s="38"/>
       <c r="Z12" s="3"/>
-      <c r="AA12" s="3"/>
+      <c r="AA12" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="17.25">
-      <c r="A13" s="31" t="s">
+      <c r="A13" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="32">
+      <c r="B13" s="34">
         <v>52.1</v>
       </c>
-      <c r="C13" s="33">
+      <c r="C13" s="35">
         <v>54.96</v>
       </c>
-      <c r="D13" s="33">
+      <c r="D13" s="35">
         <v>57.72</v>
       </c>
-      <c r="E13" s="33">
+      <c r="E13" s="35">
         <v>60.09</v>
       </c>
-      <c r="F13" s="33">
+      <c r="F13" s="35">
         <v>63.85</v>
       </c>
-      <c r="G13" s="33">
+      <c r="G13" s="35">
         <v>67.51</v>
       </c>
-      <c r="H13" s="33">
+      <c r="H13" s="35">
         <v>71.38</v>
       </c>
-      <c r="I13" s="33">
+      <c r="I13" s="35">
         <v>72.79</v>
       </c>
-      <c r="J13" s="33">
+      <c r="J13" s="35">
         <v>74.86</v>
       </c>
-      <c r="K13" s="33">
+      <c r="K13" s="35">
         <v>77.42</v>
       </c>
-      <c r="L13" s="33">
+      <c r="L13" s="35">
         <v>78.99</v>
       </c>
-      <c r="M13" s="33">
+      <c r="M13" s="35">
         <v>81.14</v>
       </c>
-      <c r="N13" s="33">
+      <c r="N13" s="35">
         <v>84.9</v>
       </c>
-      <c r="O13" s="33">
+      <c r="O13" s="35">
         <v>91.63</v>
       </c>
-      <c r="P13" s="33">
+      <c r="P13" s="35">
         <v>95.91</v>
       </c>
-      <c r="Q13" s="33">
+      <c r="Q13" s="35">
         <v>98.91</v>
       </c>
-      <c r="R13" s="33">
+      <c r="R13" s="35">
         <v>102.12</v>
       </c>
-      <c r="S13" s="33">
+      <c r="S13" s="35">
         <v>105.7</v>
       </c>
-      <c r="T13" s="33">
+      <c r="T13" s="35">
         <v>107.76</v>
       </c>
-      <c r="U13" s="33">
+      <c r="U13" s="35">
         <v>117.71</v>
       </c>
-      <c r="V13" s="33">
+      <c r="V13" s="35">
         <v>132.8</v>
       </c>
-      <c r="W13" s="33">
+      <c r="W13" s="35">
         <v>142.32</v>
       </c>
-      <c r="X13" s="33">
+      <c r="X13" s="35">
         <v>149.66</v>
       </c>
-      <c r="Y13" s="34"/>
+      <c r="Y13" s="36"/>
       <c r="Z13" s="3"/>
-      <c r="AA13" s="37"/>
+      <c r="AA13" s="39"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="17.25">
-      <c r="A14" s="27" t="s">
+      <c r="A14" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="35">
+      <c r="B14" s="37">
         <v>52.36</v>
       </c>
       <c r="C14" s="2">
@@ -1719,92 +1737,92 @@
       <c r="X14" s="2">
         <v>150.14</v>
       </c>
-      <c r="Y14" s="36"/>
+      <c r="Y14" s="38"/>
       <c r="Z14" s="3"/>
-      <c r="AA14" s="3"/>
+      <c r="AA14" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
-      <c r="A15" s="31" t="s">
+      <c r="A15" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="32">
+      <c r="B15" s="34">
         <v>52.33</v>
       </c>
-      <c r="C15" s="33">
+      <c r="C15" s="35">
         <v>55.51</v>
       </c>
-      <c r="D15" s="33">
+      <c r="D15" s="35">
         <v>58.18</v>
       </c>
-      <c r="E15" s="33">
+      <c r="E15" s="35">
         <v>60.48</v>
       </c>
-      <c r="F15" s="33">
+      <c r="F15" s="35">
         <v>64.12</v>
       </c>
-      <c r="G15" s="33">
+      <c r="G15" s="35">
         <v>68.73</v>
       </c>
-      <c r="H15" s="33">
+      <c r="H15" s="35">
         <v>71.35</v>
       </c>
-      <c r="I15" s="33">
+      <c r="I15" s="35">
         <v>72.95</v>
       </c>
-      <c r="J15" s="33">
+      <c r="J15" s="35">
         <v>75.31</v>
       </c>
-      <c r="K15" s="33">
+      <c r="K15" s="35">
         <v>77.72</v>
       </c>
-      <c r="L15" s="33">
+      <c r="L15" s="35">
         <v>79.39</v>
       </c>
-      <c r="M15" s="33">
+      <c r="M15" s="35">
         <v>81.61</v>
       </c>
-      <c r="N15" s="33">
+      <c r="N15" s="35">
         <v>85.21</v>
       </c>
-      <c r="O15" s="33">
+      <c r="O15" s="35">
         <v>92.54</v>
       </c>
-      <c r="P15" s="33">
+      <c r="P15" s="35">
         <v>96.23</v>
       </c>
-      <c r="Q15" s="33">
+      <c r="Q15" s="35">
         <v>99.31</v>
       </c>
-      <c r="R15" s="33">
+      <c r="R15" s="35">
         <v>102.71</v>
       </c>
-      <c r="S15" s="33">
+      <c r="S15" s="35">
         <v>104.97</v>
       </c>
-      <c r="T15" s="33">
+      <c r="T15" s="35">
         <v>108.78</v>
       </c>
-      <c r="U15" s="33">
+      <c r="U15" s="35">
         <v>119.31</v>
       </c>
-      <c r="V15" s="33">
+      <c r="V15" s="35">
         <v>133.78</v>
       </c>
-      <c r="W15" s="33">
+      <c r="W15" s="35">
         <v>143.38</v>
       </c>
-      <c r="X15" s="33">
+      <c r="X15" s="35">
         <v>150.3</v>
       </c>
-      <c r="Y15" s="34"/>
+      <c r="Y15" s="36"/>
       <c r="Z15" s="3"/>
-      <c r="AA15" s="3"/>
+      <c r="AA15" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="B16" s="35">
+      <c r="B16" s="37">
         <v>52.26</v>
       </c>
       <c r="C16" s="2">
@@ -1873,92 +1891,92 @@
       <c r="X16" s="2">
         <v>150.71</v>
       </c>
-      <c r="Y16" s="36"/>
+      <c r="Y16" s="38"/>
       <c r="Z16" s="3"/>
-      <c r="AA16" s="3"/>
+      <c r="AA16" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25">
-      <c r="A17" s="31" t="s">
+      <c r="A17" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="32">
+      <c r="B17" s="34">
         <v>52.42</v>
       </c>
-      <c r="C17" s="33">
+      <c r="C17" s="35">
         <v>55.51</v>
       </c>
-      <c r="D17" s="33">
+      <c r="D17" s="35">
         <v>58.21</v>
       </c>
-      <c r="E17" s="33">
+      <c r="E17" s="35">
         <v>60.96</v>
       </c>
-      <c r="F17" s="33">
+      <c r="F17" s="35">
         <v>64.14</v>
       </c>
-      <c r="G17" s="33">
+      <c r="G17" s="35">
         <v>69.19</v>
       </c>
-      <c r="H17" s="33">
+      <c r="H17" s="35">
         <v>71.35</v>
       </c>
-      <c r="I17" s="33">
+      <c r="I17" s="35">
         <v>73</v>
       </c>
-      <c r="J17" s="33">
+      <c r="J17" s="35">
         <v>75.39</v>
       </c>
-      <c r="K17" s="33">
+      <c r="K17" s="35">
         <v>77.73</v>
       </c>
-      <c r="L17" s="33">
+      <c r="L17" s="35">
         <v>79.5</v>
       </c>
-      <c r="M17" s="33">
+      <c r="M17" s="35">
         <v>81.9</v>
       </c>
-      <c r="N17" s="33">
+      <c r="N17" s="35">
         <v>85.78</v>
       </c>
-      <c r="O17" s="33">
+      <c r="O17" s="35">
         <v>92.73</v>
       </c>
-      <c r="P17" s="33">
+      <c r="P17" s="35">
         <v>96.32</v>
       </c>
-      <c r="Q17" s="33">
+      <c r="Q17" s="35">
         <v>99.3</v>
       </c>
-      <c r="R17" s="33">
+      <c r="R17" s="35">
         <v>103.03</v>
       </c>
-      <c r="S17" s="33">
+      <c r="S17" s="35">
         <v>104.96</v>
       </c>
-      <c r="T17" s="33">
+      <c r="T17" s="35">
         <v>109.62</v>
       </c>
-      <c r="U17" s="33">
+      <c r="U17" s="35">
         <v>121.5</v>
       </c>
-      <c r="V17" s="33">
+      <c r="V17" s="35">
         <v>135.39</v>
       </c>
-      <c r="W17" s="33">
+      <c r="W17" s="35">
         <v>143.67</v>
       </c>
-      <c r="X17" s="33">
+      <c r="X17" s="35">
         <v>150.99</v>
       </c>
-      <c r="Y17" s="34"/>
+      <c r="Y17" s="36"/>
       <c r="Z17" s="3"/>
-      <c r="AA17" s="3"/>
+      <c r="AA17" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="35">
+      <c r="B18" s="37">
         <v>52.53</v>
       </c>
       <c r="C18" s="2">
@@ -2027,92 +2045,92 @@
       <c r="X18" s="2">
         <v>151.48</v>
       </c>
-      <c r="Y18" s="36"/>
+      <c r="Y18" s="38"/>
       <c r="Z18" s="3"/>
-      <c r="AA18" s="3"/>
+      <c r="AA18" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
-      <c r="A19" s="31" t="s">
+      <c r="A19" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="32">
+      <c r="B19" s="34">
         <v>52.56</v>
       </c>
-      <c r="C19" s="33">
+      <c r="C19" s="35">
         <v>55.66</v>
       </c>
-      <c r="D19" s="33">
+      <c r="D19" s="35">
         <v>58.6</v>
       </c>
-      <c r="E19" s="33">
+      <c r="E19" s="35">
         <v>61.05</v>
       </c>
-      <c r="F19" s="33">
+      <c r="F19" s="35">
         <v>64.2</v>
       </c>
-      <c r="G19" s="33">
+      <c r="G19" s="35">
         <v>69.3</v>
       </c>
-      <c r="H19" s="33">
+      <c r="H19" s="35">
         <v>71.19</v>
       </c>
-      <c r="I19" s="33">
+      <c r="I19" s="35">
         <v>72.84</v>
       </c>
-      <c r="J19" s="33">
+      <c r="J19" s="35">
         <v>75.77</v>
       </c>
-      <c r="K19" s="33">
+      <c r="K19" s="35">
         <v>78.08</v>
       </c>
-      <c r="L19" s="33">
+      <c r="L19" s="35">
         <v>79.52</v>
       </c>
-      <c r="M19" s="33">
+      <c r="M19" s="35">
         <v>82.14</v>
       </c>
-      <c r="N19" s="33">
+      <c r="N19" s="35">
         <v>86.98</v>
       </c>
-      <c r="O19" s="33">
+      <c r="O19" s="35">
         <v>92.62</v>
       </c>
-      <c r="P19" s="33">
+      <c r="P19" s="35">
         <v>96.37</v>
       </c>
-      <c r="Q19" s="33">
+      <c r="Q19" s="35">
         <v>99.59</v>
       </c>
-      <c r="R19" s="33">
+      <c r="R19" s="35">
         <v>103.43</v>
       </c>
-      <c r="S19" s="33">
+      <c r="S19" s="35">
         <v>105.23</v>
       </c>
-      <c r="T19" s="33">
+      <c r="T19" s="35">
         <v>110.06</v>
       </c>
-      <c r="U19" s="33">
+      <c r="U19" s="35">
         <v>123.51</v>
       </c>
-      <c r="V19" s="33">
+      <c r="V19" s="35">
         <v>136.45</v>
       </c>
-      <c r="W19" s="33">
+      <c r="W19" s="35">
         <v>143.83</v>
       </c>
-      <c r="X19" s="33">
+      <c r="X19" s="35">
         <v>151.76</v>
       </c>
-      <c r="Y19" s="34"/>
+      <c r="Y19" s="36"/>
       <c r="Z19" s="3"/>
-      <c r="AA19" s="3"/>
+      <c r="AA19" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25">
-      <c r="A20" s="27" t="s">
+      <c r="A20" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="B20" s="35">
+      <c r="B20" s="37">
         <v>52.75</v>
       </c>
       <c r="C20" s="2">
@@ -2181,237 +2199,237 @@
       <c r="X20" s="2">
         <v>151.87</v>
       </c>
-      <c r="Y20" s="36"/>
+      <c r="Y20" s="38"/>
       <c r="Z20" s="3"/>
-      <c r="AA20" s="3"/>
+      <c r="AA20" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="17.25">
-      <c r="A21" s="38" t="s">
+      <c r="A21" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="39">
+      <c r="B21" s="41">
         <v>53.07</v>
       </c>
-      <c r="C21" s="40">
+      <c r="C21" s="42">
         <v>55.99</v>
       </c>
-      <c r="D21" s="40">
+      <c r="D21" s="42">
         <v>58.7</v>
       </c>
-      <c r="E21" s="40">
+      <c r="E21" s="42">
         <v>61.33</v>
       </c>
-      <c r="F21" s="40">
+      <c r="F21" s="42">
         <v>64.82</v>
       </c>
-      <c r="G21" s="40">
+      <c r="G21" s="42">
         <v>69.8</v>
       </c>
-      <c r="H21" s="40">
+      <c r="H21" s="42">
         <v>71.2</v>
       </c>
-      <c r="I21" s="40">
+      <c r="I21" s="42">
         <v>73.45</v>
       </c>
-      <c r="J21" s="40">
+      <c r="J21" s="42">
         <v>76.19</v>
       </c>
-      <c r="K21" s="40">
+      <c r="K21" s="42">
         <v>78.05</v>
       </c>
-      <c r="L21" s="40">
+      <c r="L21" s="42">
         <v>79.56</v>
       </c>
-      <c r="M21" s="40">
+      <c r="M21" s="42">
         <v>82.47</v>
       </c>
-      <c r="N21" s="40">
+      <c r="N21" s="42">
         <v>88.05</v>
       </c>
-      <c r="O21" s="40">
+      <c r="O21" s="42">
         <v>93.11</v>
       </c>
-      <c r="P21" s="40">
+      <c r="P21" s="42">
         <v>96.92</v>
       </c>
-      <c r="Q21" s="40">
+      <c r="Q21" s="42">
         <v>100</v>
       </c>
-      <c r="R21" s="40">
+      <c r="R21" s="42">
         <v>103.8</v>
       </c>
-      <c r="S21" s="40">
+      <c r="S21" s="42">
         <v>105.48</v>
       </c>
-      <c r="T21" s="40">
+      <c r="T21" s="42">
         <v>111.41</v>
       </c>
-      <c r="U21" s="40">
+      <c r="U21" s="42">
         <v>126.03</v>
       </c>
-      <c r="V21" s="40">
+      <c r="V21" s="42">
         <v>137.72</v>
       </c>
-      <c r="W21" s="40">
+      <c r="W21" s="42">
         <v>144.88</v>
       </c>
-      <c r="X21" s="40">
+      <c r="X21" s="42">
         <v>152.27</v>
       </c>
-      <c r="Y21" s="41"/>
+      <c r="Y21" s="43"/>
       <c r="Z21" s="3"/>
-      <c r="AA21" s="3"/>
+      <c r="AA21" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="17.25">
-      <c r="A22" s="3"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
-      <c r="M22" s="4"/>
-      <c r="N22" s="4"/>
-      <c r="O22" s="4"/>
-      <c r="P22" s="4"/>
-      <c r="Q22" s="4"/>
-      <c r="R22" s="4"/>
-      <c r="S22" s="4"/>
-      <c r="T22" s="4"/>
-      <c r="U22" s="4"/>
-      <c r="V22" s="4"/>
-      <c r="W22" s="4"/>
-      <c r="X22" s="4"/>
-      <c r="Y22" s="4"/>
+      <c r="A22" s="5"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="6"/>
+      <c r="K22" s="6"/>
+      <c r="L22" s="6"/>
+      <c r="M22" s="6"/>
+      <c r="N22" s="6"/>
+      <c r="O22" s="6"/>
+      <c r="P22" s="6"/>
+      <c r="Q22" s="6"/>
+      <c r="R22" s="6"/>
+      <c r="S22" s="6"/>
+      <c r="T22" s="6"/>
+      <c r="U22" s="6"/>
+      <c r="V22" s="6"/>
+      <c r="W22" s="6"/>
+      <c r="X22" s="6"/>
+      <c r="Y22" s="6"/>
       <c r="Z22" s="3"/>
-      <c r="AA22" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="13.5">
-      <c r="A23" s="3"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
-      <c r="L23" s="4"/>
-      <c r="M23" s="4"/>
-      <c r="N23" s="4"/>
-      <c r="O23" s="4"/>
-      <c r="P23" s="4"/>
-      <c r="Q23" s="4"/>
-      <c r="R23" s="4"/>
-      <c r="S23" s="4"/>
-      <c r="T23" s="4"/>
-      <c r="U23" s="4"/>
-      <c r="V23" s="4"/>
-      <c r="W23" s="4"/>
-      <c r="X23" s="4"/>
-      <c r="Y23" s="4"/>
+      <c r="AA22" s="4"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="17.25">
+      <c r="A23" s="5"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="6"/>
+      <c r="K23" s="6"/>
+      <c r="L23" s="6"/>
+      <c r="M23" s="6"/>
+      <c r="N23" s="6"/>
+      <c r="O23" s="6"/>
+      <c r="P23" s="6"/>
+      <c r="Q23" s="6"/>
+      <c r="R23" s="6"/>
+      <c r="S23" s="6"/>
+      <c r="T23" s="6"/>
+      <c r="U23" s="6"/>
+      <c r="V23" s="6"/>
+      <c r="W23" s="6"/>
+      <c r="X23" s="6"/>
+      <c r="Y23" s="6"/>
       <c r="Z23" s="3"/>
-      <c r="AA23" s="3"/>
+      <c r="AA23" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="17.25">
-      <c r="A24" s="42" t="s">
+      <c r="A24" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="B24" s="43"/>
-      <c r="C24" s="43"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="43"/>
-      <c r="F24" s="43"/>
-      <c r="G24" s="43"/>
-      <c r="H24" s="43"/>
-      <c r="I24" s="43"/>
-      <c r="J24" s="43"/>
-      <c r="K24" s="43"/>
-      <c r="L24" s="43"/>
-      <c r="M24" s="43"/>
-      <c r="N24" s="43"/>
-      <c r="O24" s="43"/>
-      <c r="P24" s="43"/>
-      <c r="Q24" s="43"/>
-      <c r="R24" s="43"/>
-      <c r="S24" s="43"/>
-      <c r="T24" s="19"/>
-      <c r="U24" s="19"/>
-      <c r="V24" s="19"/>
-      <c r="W24" s="19"/>
-      <c r="X24" s="19"/>
-      <c r="Y24" s="44"/>
+      <c r="B24" s="45"/>
+      <c r="C24" s="45"/>
+      <c r="D24" s="45"/>
+      <c r="E24" s="45"/>
+      <c r="F24" s="45"/>
+      <c r="G24" s="45"/>
+      <c r="H24" s="45"/>
+      <c r="I24" s="45"/>
+      <c r="J24" s="45"/>
+      <c r="K24" s="45"/>
+      <c r="L24" s="45"/>
+      <c r="M24" s="45"/>
+      <c r="N24" s="45"/>
+      <c r="O24" s="45"/>
+      <c r="P24" s="45"/>
+      <c r="Q24" s="45"/>
+      <c r="R24" s="45"/>
+      <c r="S24" s="45"/>
+      <c r="T24" s="21"/>
+      <c r="U24" s="21"/>
+      <c r="V24" s="21"/>
+      <c r="W24" s="21"/>
+      <c r="X24" s="21"/>
+      <c r="Y24" s="46"/>
       <c r="Z24" s="3"/>
-      <c r="AA24" s="3"/>
+      <c r="AA24" s="4"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="17.25">
-      <c r="A25" s="45" t="s">
+      <c r="A25" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="B25" s="46"/>
-      <c r="C25" s="46"/>
-      <c r="D25" s="46"/>
-      <c r="E25" s="46"/>
-      <c r="F25" s="46"/>
-      <c r="G25" s="46"/>
-      <c r="H25" s="46"/>
-      <c r="I25" s="46"/>
-      <c r="J25" s="46"/>
-      <c r="K25" s="46"/>
-      <c r="L25" s="46"/>
-      <c r="M25" s="46"/>
-      <c r="N25" s="46"/>
-      <c r="O25" s="46"/>
-      <c r="P25" s="46"/>
-      <c r="Q25" s="46"/>
-      <c r="R25" s="46"/>
-      <c r="S25" s="46"/>
-      <c r="T25" s="4"/>
-      <c r="U25" s="4"/>
-      <c r="V25" s="4"/>
-      <c r="W25" s="4"/>
-      <c r="X25" s="4"/>
-      <c r="Y25" s="47"/>
+      <c r="B25" s="48"/>
+      <c r="C25" s="48"/>
+      <c r="D25" s="48"/>
+      <c r="E25" s="48"/>
+      <c r="F25" s="48"/>
+      <c r="G25" s="48"/>
+      <c r="H25" s="48"/>
+      <c r="I25" s="48"/>
+      <c r="J25" s="48"/>
+      <c r="K25" s="48"/>
+      <c r="L25" s="48"/>
+      <c r="M25" s="48"/>
+      <c r="N25" s="48"/>
+      <c r="O25" s="48"/>
+      <c r="P25" s="48"/>
+      <c r="Q25" s="48"/>
+      <c r="R25" s="48"/>
+      <c r="S25" s="48"/>
+      <c r="T25" s="6"/>
+      <c r="U25" s="6"/>
+      <c r="V25" s="6"/>
+      <c r="W25" s="6"/>
+      <c r="X25" s="6"/>
+      <c r="Y25" s="49"/>
       <c r="Z25" s="3"/>
-      <c r="AA25" s="3"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="17.1">
-      <c r="A26" s="48" t="s">
+      <c r="AA25" s="4"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="17.25">
+      <c r="A26" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="B26" s="49"/>
-      <c r="C26" s="49"/>
-      <c r="D26" s="49"/>
-      <c r="E26" s="49"/>
-      <c r="F26" s="49"/>
-      <c r="G26" s="49"/>
-      <c r="H26" s="50"/>
-      <c r="I26" s="49"/>
-      <c r="J26" s="49"/>
-      <c r="K26" s="49"/>
-      <c r="L26" s="49"/>
-      <c r="M26" s="49"/>
-      <c r="N26" s="49"/>
-      <c r="O26" s="49"/>
-      <c r="P26" s="49"/>
-      <c r="Q26" s="49"/>
-      <c r="R26" s="49"/>
-      <c r="S26" s="49"/>
-      <c r="T26" s="51"/>
-      <c r="U26" s="51"/>
-      <c r="V26" s="51"/>
-      <c r="W26" s="51"/>
-      <c r="X26" s="51"/>
-      <c r="Y26" s="52"/>
+      <c r="B26" s="51"/>
+      <c r="C26" s="51"/>
+      <c r="D26" s="51"/>
+      <c r="E26" s="51"/>
+      <c r="F26" s="51"/>
+      <c r="G26" s="51"/>
+      <c r="H26" s="52"/>
+      <c r="I26" s="51"/>
+      <c r="J26" s="51"/>
+      <c r="K26" s="51"/>
+      <c r="L26" s="51"/>
+      <c r="M26" s="51"/>
+      <c r="N26" s="51"/>
+      <c r="O26" s="51"/>
+      <c r="P26" s="51"/>
+      <c r="Q26" s="51"/>
+      <c r="R26" s="51"/>
+      <c r="S26" s="51"/>
+      <c r="T26" s="53"/>
+      <c r="U26" s="53"/>
+      <c r="V26" s="53"/>
+      <c r="W26" s="53"/>
+      <c r="X26" s="53"/>
+      <c r="Y26" s="54"/>
       <c r="Z26" s="3"/>
-      <c r="AA26" s="3"/>
+      <c r="AA26" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Update datasets and data processing scripts
Refresh multiple data inputs and processed outputs and adjust processing code/tests accordingly. Changes include: updated final NAIRU dataset and various processed CSVs (brent, dane_gdp, dane_informality, dane_labor, inflation_banrep, ipc, pwt, tes), refreshed raw input files (Data_NAIRU.xlsx, PIB_CO.xlsx, IPC indices/pages), removal of obsolete raw/banrep_inflation_raw.json, and code updates in src/config.py, src/merge.py and src/sources/pwt/pwt.py. tests/test_merge.py was also updated to reflect the data/code changes.
</commit_message>
<xml_diff>
--- a/data/raw/dane/ipc_indices_raw.xlsx
+++ b/data/raw/dane/ipc_indices_raw.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\motaro\Indices\IPC\Difusión\3_Revision\7_Anexos\B. INDICES Y PONDERACIONES\Indices. Series de empalme  2003 - 2019\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\calculo\Desktop\TRABAJO ABRIL 2026\CALCULO ABRIL\10. PRODUCTO ANEXO VARIACIONES\Indices. Series de empalme  2003 - 2019\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D621B227-09BA-4A5A-92FE-EF00C6B5F0A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFF4C324-240B-47F1-A1A8-11143DAD5C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,9 +27,6 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -129,7 +126,7 @@
 2003 - 2026</t>
   </si>
   <si>
-    <t>Actualizado el 9 de Abril de 2026</t>
+    <t>Actualizado el 8 de Mayo de 2026</t>
   </si>
 </sst>
 </file>
@@ -2212,7 +2209,9 @@
       <c r="X13" s="14">
         <v>149.66</v>
       </c>
-      <c r="Y13" s="26"/>
+      <c r="Y13" s="26">
+        <v>158.16999999999999</v>
+      </c>
       <c r="AA13" s="49"/>
     </row>
     <row r="14" spans="1:27" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2">
@@ -2917,6 +2916,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010027BDBDF69F845F4383C93D67CEBAFF04" ma:contentTypeVersion="4" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="0ea007cbf4cb5b5cc813a7650d64ca58">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb0b624f-ae06-4913-a28b-bf5d24a61ccb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8b65969171b7152b51da7f3e00aa75fb" ns2:_="">
     <xsd:import namespace="bb0b624f-ae06-4913-a28b-bf5d24a61ccb"/>
@@ -3060,22 +3074,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A6CEC6C9-CA48-4E93-BC99-F210F33FD8FB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="bb0b624f-ae06-4913-a28b-bf5d24a61ccb"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D72D454-867A-47C4-AB39-812B39DB7663}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85115342-A464-41ED-B238-9E002ED72CDD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3091,28 +3114,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D72D454-867A-47C4-AB39-812B39DB7663}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A6CEC6C9-CA48-4E93-BC99-F210F33FD8FB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="bb0b624f-ae06-4913-a28b-bf5d24a61ccb"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix(viog/kalman): UCM en log(PIB) + start_params en cuenca económica
- Aplicar UCM a log(PIB) en vez de niveles (equivalente a Stata 'ucm lnpib')
- Reconvertir tendencia: trend_kalman = exp(result.level.smoothed)
- Inicializar sigma2.cycle = Var(ΔlnPIB), rho = 0.70, freq = 2pi/32
  para evitar convergencia al máximo local degenerado (sigma2.cycle -> 0)
- La función de log-verosimilitud tiene dos máximos locales:
    (a) Degenerado (llf≈296): sigma2.cycle→0, gap≈0  ← antes
    (b) Económico  (llf≈290): sigma2.cycle≈Var(ΔlnPIB) ← ahora (= Stata)
- Actualizar notebook VIOG (3).ipynb con la misma corrección

Resultados Colombia vs Stata:
  std(gap_kalman): 0.0290 Python vs 0.0221 Stata (antes: 0.0892)
  COVID 2020Q2:   -19.3% Python vs -18.8% Stata (antes: -10.8%)
  burn-in 1994:   razonable  (antes: +75.6%)
</commit_message>
<xml_diff>
--- a/data/raw/dane/ipc_indices_raw.xlsx
+++ b/data/raw/dane/ipc_indices_raw.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\calculo\Desktop\TRABAJO ABRIL 2026\CALCULO ABRIL\10. PRODUCTO ANEXO VARIACIONES\Indices. Series de empalme  2003 - 2019\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\calculo\Desktop\RO-IPC-07-26\Producción\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFF4C324-240B-47F1-A1A8-11143DAD5C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{51C2A6AD-C825-4B7F-A946-B2E3C61CF4B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -126,7 +126,7 @@
 2003 - 2026</t>
   </si>
   <si>
-    <t>Actualizado el 8 de Mayo de 2026</t>
+    <t>Actualizado el 7 de Julio de 2026</t>
   </si>
 </sst>
 </file>
@@ -1649,7 +1649,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AA26"/>
+  <dimension ref="A1:AB26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="14.25" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.42578125" style="8" customWidth="1"/>
@@ -1658,7 +1658,7 @@
     <col min="26" max="16384" width="11.42578125" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="6" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:28" s="6" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="55"/>
       <c r="B1" s="55"/>
       <c r="C1" s="55"/>
@@ -1685,8 +1685,8 @@
       <c r="X1" s="55"/>
       <c r="Y1" s="55"/>
     </row>
-    <row r="2" spans="1:27" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2"/>
-    <row r="3" spans="1:27" s="6" customFormat="1" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:28" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2"/>
+    <row r="3" spans="1:28" s="6" customFormat="1" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="56" t="s">
         <v>15</v>
       </c>
@@ -1715,7 +1715,7 @@
       <c r="X3" s="56"/>
       <c r="Y3" s="56"/>
     </row>
-    <row r="4" spans="1:27" s="6" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:28" s="6" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="56"/>
       <c r="B4" s="56"/>
       <c r="C4" s="56"/>
@@ -1742,7 +1742,7 @@
       <c r="X4" s="56"/>
       <c r="Y4" s="56"/>
     </row>
-    <row r="5" spans="1:27" s="6" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:28" s="6" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="57" t="s">
         <v>17</v>
       </c>
@@ -1771,8 +1771,8 @@
       <c r="X5" s="58"/>
       <c r="Y5" s="58"/>
     </row>
-    <row r="6" spans="1:27" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2"/>
-    <row r="7" spans="1:27" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:28" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2"/>
+    <row r="7" spans="1:28" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="18"/>
       <c r="C7" s="18"/>
@@ -1799,7 +1799,7 @@
       <c r="X7" s="18"/>
       <c r="Y7" s="18"/>
     </row>
-    <row r="8" spans="1:27" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:28" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -1828,7 +1828,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:27" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:28" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>14</v>
       </c>
@@ -1905,7 +1905,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="10" spans="1:27" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:28" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>1</v>
       </c>
@@ -1982,7 +1982,7 @@
         <v>154.07</v>
       </c>
     </row>
-    <row r="11" spans="1:27" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:28" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>2</v>
       </c>
@@ -2059,7 +2059,7 @@
         <v>155.72999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:27" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:28" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>3</v>
       </c>
@@ -2136,7 +2136,7 @@
         <v>156.94</v>
       </c>
     </row>
-    <row r="13" spans="1:27" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:28" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>4</v>
       </c>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="AA13" s="49"/>
     </row>
-    <row r="14" spans="1:27" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:28" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>5</v>
       </c>
@@ -2287,9 +2287,11 @@
       <c r="X14" s="13">
         <v>150.13999999999999</v>
       </c>
-      <c r="Y14" s="39"/>
+      <c r="Y14" s="39">
+        <v>158.91</v>
+      </c>
     </row>
-    <row r="15" spans="1:27" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:28" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>6</v>
       </c>
@@ -2362,9 +2364,12 @@
       <c r="X15" s="14">
         <v>150.30000000000001</v>
       </c>
-      <c r="Y15" s="26"/>
+      <c r="Y15" s="26">
+        <v>159.53</v>
+      </c>
+      <c r="AB15" s="49"/>
     </row>
-    <row r="16" spans="1:27" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:28" s="6" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>7</v>
       </c>
@@ -2922,15 +2927,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010027BDBDF69F845F4383C93D67CEBAFF04" ma:contentTypeVersion="4" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="0ea007cbf4cb5b5cc813a7650d64ca58">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb0b624f-ae06-4913-a28b-bf5d24a61ccb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8b65969171b7152b51da7f3e00aa75fb" ns2:_="">
     <xsd:import namespace="bb0b624f-ae06-4913-a28b-bf5d24a61ccb"/>
@@ -3074,6 +3070,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A6CEC6C9-CA48-4E93-BC99-F210F33FD8FB}">
   <ds:schemaRefs>
@@ -3091,14 +3096,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D72D454-867A-47C4-AB39-812B39DB7663}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85115342-A464-41ED-B238-9E002ED72CDD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3114,4 +3111,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D72D454-867A-47C4-AB39-812B39DB7663}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>